<commit_message>
add research results pagination and DOI links
</commit_message>
<xml_diff>
--- a/frontend/data-source/publications.xlsx
+++ b/frontend/data-source/publications.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="学术论文" sheetId="1" r:id="R93aa99688a344d17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="学术论文" sheetId="1" r:id="R94a918264e60434a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -704,7 +704,7 @@
         <x:v>Enhanced Prompting Framework for Code Summarization with Large Language Models</x:v>
       </x:c>
       <x:c r="D13" s="12" t="str">
-        <x:v>https://scholar.google.com/citations?view_op=view_citation&amp;hl=zh-CN&amp;user=S3Rd5TgAAAAJ&amp;cstart=20&amp;pagesize=80&amp;sortby=pubdate&amp;citation_for_view=S3Rd5TgAAAAJ:1lhNe0rCu4AC</x:v>
+        <x:v>https://doi.org/10.1145/3728949</x:v>
       </x:c>
       <x:c r="E13" s="12" t="str">
         <x:v>published</x:v>
@@ -791,7 +791,7 @@
         <x:v>Hidden Backdoor Attack against Neural Code Search Models</x:v>
       </x:c>
       <x:c r="D16" s="12" t="str">
-        <x:v>https://scholar.google.com/citations?view_op=view_citation&amp;hl=zh-CN&amp;user=HQWxCnkAAAAJ&amp;cstart=20&amp;pagesize=80&amp;sortby=pubdate&amp;citation_for_view=HQWxCnkAAAAJ:IwGqIHSOC8kC</x:v>
+        <x:v>https://doi.org/10.1145/3774421</x:v>
       </x:c>
       <x:c r="E16" s="12" t="str">
         <x:v>published</x:v>
@@ -965,7 +965,7 @@
         <x:v>pFedLVM: A Large Vision Model (LVM)-Driven and Latent Feature-Based Personalized Federated Learning Framework in Autonomous Driving</x:v>
       </x:c>
       <x:c r="D22" s="12" t="str">
-        <x:v>https://scholar.google.com/citations?view_op=view_citation&amp;hl=zh-CN&amp;user=HQWxCnkAAAAJ&amp;cstart=20&amp;pagesize=80&amp;sortby=pubdate&amp;citation_for_view=HQWxCnkAAAAJ:5McdzzY_mmwC</x:v>
+        <x:v>https://doi.org/10.1109/TITS.2025.3581939</x:v>
       </x:c>
       <x:c r="E22" s="12" t="str">
         <x:v>published</x:v>
@@ -994,7 +994,7 @@
         <x:v>Pre-trained Model-based Actionable Warning Identification: A Feasibility Study</x:v>
       </x:c>
       <x:c r="D23" s="12" t="str">
-        <x:v>https://scholar.google.com/citations?view_op=view_citation&amp;hl=zh-CN&amp;user=S3Rd5TgAAAAJ&amp;cstart=20&amp;pagesize=80&amp;sortby=pubdate&amp;citation_for_view=S3Rd5TgAAAAJ:rmuvC79q63oC</x:v>
+        <x:v>https://doi.org/10.1145/3777369</x:v>
       </x:c>
       <x:c r="E23" s="12" t="str">
         <x:v>published</x:v>
@@ -1197,7 +1197,7 @@
         <x:v>Tightening Robustness Verification of MaxPool-based Neural Networks via Minimizing the Over-Approximation Zone</x:v>
       </x:c>
       <x:c r="D30" s="12" t="str">
-        <x:v>https://scholar.google.com/citations?view_op=view_citation&amp;hl=zh-CN&amp;user=HQWxCnkAAAAJ&amp;cstart=20&amp;pagesize=80&amp;sortby=pubdate&amp;citation_for_view=HQWxCnkAAAAJ:HkunuPqSaCsC</x:v>
+        <x:v>https://doi.org/10.1109/CVPR52734.2025.01927</x:v>
       </x:c>
       <x:c r="E30" s="12" t="str">
         <x:v>published</x:v>
@@ -1226,7 +1226,7 @@
         <x:v>Understanding LLM-Centric Challenges for Deep Learning Frameworks: An Empirical Analysis</x:v>
       </x:c>
       <x:c r="D31" s="12" t="str">
-        <x:v>https://scholar.google.com/citations?view_op=view_citation&amp;hl=zh-CN&amp;user=HQWxCnkAAAAJ&amp;cstart=20&amp;pagesize=80&amp;sortby=pubdate&amp;citation_for_view=HQWxCnkAAAAJ:YIdQ7BAI8VoC</x:v>
+        <x:v>https://doi.org/10.1145/3821532</x:v>
       </x:c>
       <x:c r="E31" s="12" t="str">
         <x:v>published</x:v>
@@ -1313,7 +1313,7 @@
         <x:v>A Survey of Learning-based Method Name Prediction</x:v>
       </x:c>
       <x:c r="D34" s="12" t="str">
-        <x:v>https://scholar.google.com/citations?view_op=view_citation&amp;hl=zh-CN&amp;user=S3Rd5TgAAAAJ&amp;cstart=100&amp;pagesize=100&amp;sortby=pubdate&amp;citation_for_view=S3Rd5TgAAAAJ:7wO8s98CvbsC</x:v>
+        <x:v>https://doi.org/10.1145/3771999</x:v>
       </x:c>
       <x:c r="E34" s="12" t="str">
         <x:v>published</x:v>
@@ -1371,7 +1371,7 @@
         <x:v>A Systematic Literature Review on Large Language Models for Automated Program Repair</x:v>
       </x:c>
       <x:c r="D36" s="12" t="str">
-        <x:v>https://scholar.google.com/citations?view_op=view_citation&amp;hl=zh-CN&amp;user=S3Rd5TgAAAAJ&amp;cstart=100&amp;pagesize=100&amp;sortby=pubdate&amp;citation_for_view=S3Rd5TgAAAAJ:bz8QjSJIRt4C</x:v>
+        <x:v>https://doi.org/10.1145/3799693</x:v>
       </x:c>
       <x:c r="E36" s="12" t="str">
         <x:v>published</x:v>
@@ -1748,7 +1748,7 @@
         <x:v>Machine Translation Testing via Syntactic Tree Pruning</x:v>
       </x:c>
       <x:c r="D49" s="12" t="str">
-        <x:v>https://scholar.google.com/citations?view_op=view_citation&amp;hl=zh-CN&amp;user=S3Rd5TgAAAAJ&amp;cstart=20&amp;pagesize=80&amp;sortby=pubdate&amp;citation_for_view=S3Rd5TgAAAAJ:5qfkUJPXOUwC</x:v>
+        <x:v>https://doi.org/10.1145/3640329</x:v>
       </x:c>
       <x:c r="E49" s="12" t="str">
         <x:v>published</x:v>
@@ -1980,7 +1980,7 @@
         <x:v>Test Case Generation for Ethereum Smart Contracts Based on Cross-Contract Data Flow Analysis</x:v>
       </x:c>
       <x:c r="D57" s="12" t="str">
-        <x:v>https://scholar.google.com/citations?view_op=view_citation&amp;hl=zh-CN&amp;user=HQWxCnkAAAAJ&amp;cstart=20&amp;pagesize=80&amp;sortby=pubdate&amp;citation_for_view=HQWxCnkAAAAJ:Qy-rCirNo-8C</x:v>
+        <x:v>https://doi.org/10.1109/TR.2024.3494798</x:v>
       </x:c>
       <x:c r="E57" s="12" t="str">
         <x:v>published</x:v>
@@ -2096,7 +2096,7 @@
         <x:v>An Empirical Study of Class Rebalancing Methods for Actionable Warning Identification</x:v>
       </x:c>
       <x:c r="D61" s="12" t="str">
-        <x:v>https://scholar.google.com/citations?view_op=view_citation&amp;hl=zh-CN&amp;user=S3Rd5TgAAAAJ&amp;cstart=100&amp;pagesize=100&amp;sortby=pubdate&amp;citation_for_view=S3Rd5TgAAAAJ:XD-gHx7UXLsC</x:v>
+        <x:v>https://doi.org/10.1109/TR.2023.3234982</x:v>
       </x:c>
       <x:c r="E61" s="12" t="str">
         <x:v>published</x:v>
@@ -2241,7 +2241,7 @@
         <x:v>Deep learning framework testing via hierarchical and heuristic model generation</x:v>
       </x:c>
       <x:c r="D66" s="12" t="str">
-        <x:v>https://scholar.google.com/citations?view_op=view_citation&amp;hl=zh-CN&amp;user=S3Rd5TgAAAAJ&amp;cstart=100&amp;pagesize=100&amp;sortby=pubdate&amp;citation_for_view=S3Rd5TgAAAAJ:0KyAp5RtaNEC</x:v>
+        <x:v>https://doi.org/10.1016/j.jss.2023.111681</x:v>
       </x:c>
       <x:c r="E66" s="12" t="str">
         <x:v>published</x:v>
@@ -2444,7 +2444,7 @@
         <x:v>Pre-Trained Model-Based Automated Software Vulnerability Repair: How Far are We?</x:v>
       </x:c>
       <x:c r="D73" s="12" t="str">
-        <x:v>https://scholar.google.com/citations?view_op=view_citation&amp;hl=zh-CN&amp;user=HQWxCnkAAAAJ&amp;cstart=100&amp;pagesize=100&amp;sortby=pubdate&amp;citation_for_view=HQWxCnkAAAAJ:WsFh9Szeq2wC</x:v>
+        <x:v>https://doi.org/10.1109/TDSC.2023.3308897</x:v>
       </x:c>
       <x:c r="E73" s="12" t="str">
         <x:v>published</x:v>
@@ -2502,7 +2502,7 @@
         <x:v>Test Report Generation for Android App Testing Via Heterogeneous Data Analysis</x:v>
       </x:c>
       <x:c r="D75" s="12" t="str">
-        <x:v>https://scholar.google.com/citations?view_op=view_citation&amp;hl=zh-CN&amp;user=S3Rd5TgAAAAJ&amp;cstart=100&amp;pagesize=100&amp;sortby=pubdate&amp;citation_for_view=S3Rd5TgAAAAJ:t7zJ5fGR-2UC</x:v>
+        <x:v>https://doi.org/10.1109/TSE.2023.3237247</x:v>
       </x:c>
       <x:c r="E75" s="12" t="str">
         <x:v>published</x:v>
@@ -2560,7 +2560,7 @@
         <x:v>ASRTest: automated testing for deep-neural-network-driven speech recognition systems</x:v>
       </x:c>
       <x:c r="D77" s="12" t="str">
-        <x:v>https://scholar.google.com/citations?view_op=view_citation&amp;hl=zh-CN&amp;user=HQWxCnkAAAAJ&amp;cstart=100&amp;pagesize=100&amp;sortby=pubdate&amp;citation_for_view=HQWxCnkAAAAJ:4pF9x-cDGsoC</x:v>
+        <x:v>https://doi.org/10.1145/3533767.3534391</x:v>
       </x:c>
       <x:c r="E77" s="12" t="str">
         <x:v>published</x:v>
@@ -2589,7 +2589,7 @@
         <x:v>CIRCLE: continual repair across programming languages</x:v>
       </x:c>
       <x:c r="D78" s="12" t="str">
-        <x:v>https://scholar.google.com/citations?view_op=view_citation&amp;hl=zh-CN&amp;user=S3Rd5TgAAAAJ&amp;cstart=100&amp;pagesize=100&amp;sortby=pubdate&amp;citation_for_view=S3Rd5TgAAAAJ:hkOj_22Ku90C</x:v>
+        <x:v>https://doi.org/10.1145/3533767.3534219</x:v>
       </x:c>
       <x:c r="E78" s="12" t="str">
         <x:v>published</x:v>
@@ -2618,7 +2618,7 @@
         <x:v>Classifying crowdsourced mobile test reports with image features: An empirical study</x:v>
       </x:c>
       <x:c r="D79" s="12" t="str">
-        <x:v>https://scholar.google.com/citations?view_op=view_citation&amp;hl=zh-CN&amp;user=HQWxCnkAAAAJ&amp;cstart=100&amp;pagesize=100&amp;sortby=pubdate&amp;citation_for_view=HQWxCnkAAAAJ:S0RksyIsHSIC</x:v>
+        <x:v>https://doi.org/10.1016/j.jss.2021.111121</x:v>
       </x:c>
       <x:c r="E79" s="12" t="str">
         <x:v>published</x:v>
@@ -2647,7 +2647,7 @@
         <x:v>Code Search based on Context-aware Code Translation</x:v>
       </x:c>
       <x:c r="D80" s="12" t="str">
-        <x:v>https://scholar.google.com/citations?view_op=view_citation&amp;hl=zh-CN&amp;user=S3Rd5TgAAAAJ&amp;cstart=100&amp;pagesize=100&amp;sortby=pubdate&amp;citation_for_view=S3Rd5TgAAAAJ:oNZyr7d5Mn4C</x:v>
+        <x:v>https://doi.org/10.1145/3510003.3510140</x:v>
       </x:c>
       <x:c r="E80" s="12" t="str">
         <x:v>published</x:v>
@@ -2676,7 +2676,7 @@
         <x:v>DeepState: Selecting Test Suites to Enhance the Robustness of Recurrent Neural Networks</x:v>
       </x:c>
       <x:c r="D81" s="12" t="str">
-        <x:v>https://scholar.google.com/citations?view_op=view_citation&amp;hl=zh-CN&amp;user=HQWxCnkAAAAJ&amp;cstart=100&amp;pagesize=100&amp;sortby=pubdate&amp;citation_for_view=HQWxCnkAAAAJ:9fRKRCJz75UC</x:v>
+        <x:v>https://doi.org/10.1145/3510003.3510231</x:v>
       </x:c>
       <x:c r="E81" s="12" t="str">
         <x:v>published</x:v>
@@ -2734,7 +2734,7 @@
         <x:v>Leveraging Android Automated Testing to Assist Crowdsourced Testing</x:v>
       </x:c>
       <x:c r="D83" s="12" t="str">
-        <x:v>https://scholar.google.com/citations?view_op=view_citation&amp;hl=zh-CN&amp;user=S3Rd5TgAAAAJ&amp;cstart=100&amp;pagesize=100&amp;sortby=pubdate&amp;citation_for_view=S3Rd5TgAAAAJ:tzM49s52ZIMC</x:v>
+        <x:v>https://doi.org/10.1109/TSE.2022.3216879</x:v>
       </x:c>
       <x:c r="E83" s="12" t="str">
         <x:v>published</x:v>
@@ -2763,7 +2763,7 @@
         <x:v>LiRTest: augmenting LiDAR point clouds for automated testing of autonomous driving systems</x:v>
       </x:c>
       <x:c r="D84" s="12" t="str">
-        <x:v>https://scholar.google.com/citations?view_op=view_citation&amp;hl=zh-CN&amp;user=HQWxCnkAAAAJ&amp;cstart=100&amp;pagesize=100&amp;sortby=pubdate&amp;citation_for_view=HQWxCnkAAAAJ:z-B63o8J19IC</x:v>
+        <x:v>https://doi.org/10.1145/3533767.3534397</x:v>
       </x:c>
       <x:c r="E84" s="12" t="str">
         <x:v>published</x:v>
@@ -2879,7 +2879,7 @@
         <x:v>RULER: discriminative and iterative adversarial training for deep neural network fairness</x:v>
       </x:c>
       <x:c r="D88" s="12" t="str">
-        <x:v>https://scholar.google.com/citations?view_op=view_citation&amp;hl=zh-CN&amp;user=S3Rd5TgAAAAJ&amp;cstart=100&amp;pagesize=100&amp;sortby=pubdate&amp;citation_for_view=S3Rd5TgAAAAJ:7T2F9Uy0os0C</x:v>
+        <x:v>https://doi.org/10.1145/3540250.3549169</x:v>
       </x:c>
       <x:c r="E88" s="12" t="str">
         <x:v>published</x:v>
@@ -2937,7 +2937,7 @@
         <x:v>SemCluster: a semi-supervised clustering tool for crowdsourced test reports with deep image understanding</x:v>
       </x:c>
       <x:c r="D90" s="12" t="str">
-        <x:v>https://scholar.google.com/citations?view_op=view_citation&amp;hl=zh-CN&amp;user=HQWxCnkAAAAJ&amp;cstart=100&amp;pagesize=100&amp;sortby=pubdate&amp;citation_for_view=HQWxCnkAAAAJ:dHRcJqc9SEQC</x:v>
+        <x:v>https://doi.org/10.1145/3540250.3558933</x:v>
       </x:c>
       <x:c r="E90" s="12" t="str">
         <x:v>published</x:v>
@@ -3024,7 +3024,7 @@
         <x:v>Test case prioritization using partial attention</x:v>
       </x:c>
       <x:c r="D93" s="12" t="str">
-        <x:v>https://scholar.google.com/citations?view_op=view_citation&amp;hl=zh-CN&amp;user=S3Rd5TgAAAAJ&amp;cstart=100&amp;pagesize=100&amp;sortby=pubdate&amp;citation_for_view=S3Rd5TgAAAAJ:PR6Y55bgFSsC</x:v>
+        <x:v>https://doi.org/10.1016/j.jss.2022.111419</x:v>
       </x:c>
       <x:c r="E93" s="12" t="str">
         <x:v>published</x:v>
@@ -3082,7 +3082,7 @@
         <x:v>UniRLTest: universal platform-independent testing with reinforcement learning via image understanding</x:v>
       </x:c>
       <x:c r="D95" s="12" t="str">
-        <x:v>https://scholar.google.com/citations?view_op=view_citation&amp;hl=zh-CN&amp;user=HQWxCnkAAAAJ&amp;cstart=100&amp;pagesize=100&amp;sortby=pubdate&amp;citation_for_view=HQWxCnkAAAAJ:C-SEpTPhZ1wC</x:v>
+        <x:v>https://doi.org/10.1145/3533767.3543292</x:v>
       </x:c>
       <x:c r="E95" s="12" t="str">
         <x:v>published</x:v>
@@ -3111,7 +3111,7 @@
         <x:v>DialTest: automated testing for recurrent-neural-network-driven dialogue systems</x:v>
       </x:c>
       <x:c r="D96" s="12" t="str">
-        <x:v>https://scholar.google.com/citations?view_op=view_citation&amp;hl=zh-CN&amp;user=HQWxCnkAAAAJ&amp;cstart=100&amp;pagesize=100&amp;sortby=pubdate&amp;citation_for_view=HQWxCnkAAAAJ:Np1obAXpBq8C</x:v>
+        <x:v>https://doi.org/10.1145/3460319.3464829</x:v>
       </x:c>
       <x:c r="E96" s="12" t="str">
         <x:v>published</x:v>
@@ -3140,7 +3140,7 @@
         <x:v>Duo: Differential Fuzzing for Deep Learning Operators</x:v>
       </x:c>
       <x:c r="D97" s="12" t="str">
-        <x:v>https://scholar.google.com/citations?view_op=view_citation&amp;hl=zh-CN&amp;user=HQWxCnkAAAAJ&amp;cstart=100&amp;pagesize=100&amp;sortby=pubdate&amp;citation_for_view=HQWxCnkAAAAJ:qt-6tCTBDsQC</x:v>
+        <x:v>https://doi.org/10.1109/TR.2021.3107165</x:v>
       </x:c>
       <x:c r="E97" s="12" t="str">
         <x:v>published</x:v>
@@ -3169,7 +3169,7 @@
         <x:v>Graph-based Fuzz Testing for Deep Learning Inference Engines</x:v>
       </x:c>
       <x:c r="D98" s="12" t="str">
-        <x:v>https://scholar.google.com/citations?view_op=view_citation&amp;hl=zh-CN&amp;user=HQWxCnkAAAAJ&amp;cstart=100&amp;pagesize=100&amp;sortby=pubdate&amp;citation_for_view=HQWxCnkAAAAJ:dT4-KZ621vcC</x:v>
+        <x:v>https://doi.org/10.1109/ICSE43902.2021.00037</x:v>
       </x:c>
       <x:c r="E98" s="12" t="str">
         <x:v>published</x:v>
@@ -3198,7 +3198,7 @@
         <x:v>Guest Editorial: A Retrospective of Special Sections on Software Testing and Program Analysis</x:v>
       </x:c>
       <x:c r="D99" s="12" t="str">
-        <x:v>https://scholar.google.com/citations?view_op=view_citation&amp;hl=zh-CN&amp;user=HQWxCnkAAAAJ&amp;cstart=100&amp;pagesize=100&amp;sortby=pubdate&amp;citation_for_view=HQWxCnkAAAAJ:wTekDMGr9GkC</x:v>
+        <x:v>https://doi.org/10.1109/TR.2021.3083375</x:v>
       </x:c>
       <x:c r="E99" s="12" t="str">
         <x:v>published</x:v>
@@ -3227,7 +3227,7 @@
         <x:v>Layout and Image Recognition Driving Cross-Platform Automated Mobile Testing</x:v>
       </x:c>
       <x:c r="D100" s="12" t="str">
-        <x:v>https://scholar.google.com/citations?view_op=view_citation&amp;hl=zh-CN&amp;user=S3Rd5TgAAAAJ&amp;cstart=100&amp;pagesize=100&amp;sortby=pubdate&amp;citation_for_view=S3Rd5TgAAAAJ:1qzjygNMrQYC</x:v>
+        <x:v>https://doi.org/10.1109/ICSE43902.2021.00139</x:v>
       </x:c>
       <x:c r="E100" s="12" t="str">
         <x:v>published</x:v>
@@ -3256,7 +3256,7 @@
         <x:v>Predoo: precision testing of deep learning operators</x:v>
       </x:c>
       <x:c r="D101" s="12" t="str">
-        <x:v>https://scholar.google.com/citations?view_op=view_citation&amp;hl=zh-CN&amp;user=HQWxCnkAAAAJ&amp;cstart=100&amp;pagesize=100&amp;sortby=pubdate&amp;citation_for_view=HQWxCnkAAAAJ:DrOLxFoABAwC</x:v>
+        <x:v>https://doi.org/10.1145/3460319.3464843</x:v>
       </x:c>
       <x:c r="E101" s="12" t="str">
         <x:v>published</x:v>
@@ -3285,7 +3285,7 @@
         <x:v>Prioritize Crowdsourced Test Reports via Deep Screenshot Understanding</x:v>
       </x:c>
       <x:c r="D102" s="12" t="str">
-        <x:v>https://scholar.google.com/citations?view_op=view_citation&amp;hl=zh-CN&amp;user=HQWxCnkAAAAJ&amp;cstart=100&amp;pagesize=100&amp;sortby=pubdate&amp;citation_for_view=HQWxCnkAAAAJ:JoHZYnTS1h4C</x:v>
+        <x:v>https://doi.org/10.1109/ICSE43902.2021.00090</x:v>
       </x:c>
       <x:c r="E102" s="12" t="str">
         <x:v>published</x:v>
@@ -3314,7 +3314,7 @@
         <x:v>Smart Contract Development: Challenges and Opportunities</x:v>
       </x:c>
       <x:c r="D103" s="12" t="str">
-        <x:v>https://scholar.google.com/citations?view_op=view_citation&amp;hl=zh-CN&amp;user=HQWxCnkAAAAJ&amp;cstart=100&amp;pagesize=100&amp;sortby=pubdate&amp;citation_for_view=HQWxCnkAAAAJ:TewouNez5YAC</x:v>
+        <x:v>https://doi.org/10.1109/TSE.2019.2942301</x:v>
       </x:c>
       <x:c r="E103" s="12" t="str">
         <x:v>published</x:v>
@@ -3343,7 +3343,7 @@
         <x:v>TauMed: test augmentation of deep learning in medical diagnosis</x:v>
       </x:c>
       <x:c r="D104" s="12" t="str">
-        <x:v>https://scholar.google.com/citations?view_op=view_citation&amp;hl=zh-CN&amp;user=HQWxCnkAAAAJ&amp;cstart=100&amp;pagesize=100&amp;sortby=pubdate&amp;citation_for_view=HQWxCnkAAAAJ:n8FNryW2AHIC</x:v>
+        <x:v>https://doi.org/10.1145/3460319.3469080</x:v>
       </x:c>
       <x:c r="E104" s="12" t="str">
         <x:v>published</x:v>
@@ -3371,7 +3371,9 @@
       <x:c r="C105" s="12" t="str">
         <x:v>Crowdsourced Requirements Generation for Automatic Testing via Knowledge Graph</x:v>
       </x:c>
-      <x:c r="D105" s="12" t="str"/>
+      <x:c r="D105" s="12" t="str">
+        <x:v>https://doi.org/10.1145/3395363.3404363</x:v>
+      </x:c>
       <x:c r="E105" s="12" t="str">
         <x:v>published</x:v>
       </x:c>
@@ -3485,7 +3487,9 @@
       <x:c r="C109" s="12" t="str">
         <x:v>Jones, Zhenyu Chen. Clustering Crowdsourced Test Reports of Mobile Applications Using Image Understanding</x:v>
       </x:c>
-      <x:c r="D109" s="12" t="str"/>
+      <x:c r="D109" s="12" t="str">
+        <x:v>https://doi.org/10.1109/TSE.2020.3017514</x:v>
+      </x:c>
       <x:c r="E109" s="12" t="str">
         <x:v>published</x:v>
       </x:c>
@@ -3541,7 +3545,9 @@
       <x:c r="C111" s="12" t="str">
         <x:v>TauJud: Test Augmentation of Machine Learning in Judicial Documents</x:v>
       </x:c>
-      <x:c r="D111" s="12" t="str"/>
+      <x:c r="D111" s="12" t="str">
+        <x:v>https://doi.org/10.1145/3395363.3404364</x:v>
+      </x:c>
       <x:c r="E111" s="12" t="str">
         <x:v>published</x:v>
       </x:c>
@@ -3916,7 +3922,9 @@
       <x:c r="C124" s="12" t="str">
         <x:v>How practitioners perceive automated bug report management techniques</x:v>
       </x:c>
-      <x:c r="D124" s="12" t="str"/>
+      <x:c r="D124" s="12" t="str">
+        <x:v>https://doi.org/10.1109/TSE.2018.2870414</x:v>
+      </x:c>
       <x:c r="E124" s="12" t="str">
         <x:v>published</x:v>
       </x:c>
@@ -3943,7 +3951,9 @@
       <x:c r="C125" s="12" t="str">
         <x:v>Eric Wong, Zhenyu Chen, Yabin Wang. Effective software fault localization using predicted execution results</x:v>
       </x:c>
-      <x:c r="D125" s="12" t="str"/>
+      <x:c r="D125" s="12" t="str">
+        <x:v>https://doi.org/10.1007/s11219-015-9295-1</x:v>
+      </x:c>
       <x:c r="E125" s="12" t="str">
         <x:v>published</x:v>
       </x:c>
@@ -4203,7 +4213,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4010d504d97f41a6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3861cb8235c7446c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>